<commit_message>
Backup PMPUy: Registro de varamientos.xlsx
</commit_message>
<xml_diff>
--- a/Respaldo_PMPUy/Formulario (no editar manualmente)/Registro de varamientos.xlsx
+++ b/Respaldo_PMPUy/Formulario (no editar manualmente)/Registro de varamientos.xlsx
@@ -58,25 +58,25 @@
     <t>Tramo 2</t>
   </si>
   <si>
-    <t>Sector E</t>
-  </si>
-  <si>
-    <t>-34.82629827326442, -54.61928315475239</t>
-  </si>
-  <si>
-    <t>Esqueleto</t>
-  </si>
-  <si>
-    <t>Tortuga Cabezona</t>
+    <t>Sector D</t>
+  </si>
+  <si>
+    <t>-34.84066585786591, -54.666520737583255</t>
+  </si>
+  <si>
+    <t>Carcasa</t>
+  </si>
+  <si>
+    <t>pinnipedo</t>
   </si>
   <si>
     <t>ref test</t>
   </si>
   <si>
-    <t>https://drive.google.com/open?id=1O8fg-aa0qQgBg3BP5IoDPVknz0SLhbuO</t>
-  </si>
-  <si>
-    <t>notas test</t>
+    <t>https://drive.google.com/open?id=1Wa7hU-cZPtndJT0jQ5atf94mXkn2VNAn</t>
+  </si>
+  <si>
+    <t>ref notas</t>
   </si>
 </sst>
 </file>
@@ -509,7 +509,7 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4">
-        <v>46114.474706099536</v>
+        <v>46114.65558759259</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
@@ -527,13 +527,13 @@
         <v>46114.0</v>
       </c>
       <c r="G2" s="8">
-        <v>0.4743055555591127</v>
+        <v>0.6548611111065838</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>17</v>
       </c>
       <c r="I2" s="5">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>18</v>

</xml_diff>